<commit_message>
Actualiza el libro: tabla dinámica refrescada con los datos finales
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015rk3UQvdsaFRzUdBW3ikUa
</commit_message>
<xml_diff>
--- a/libro/Tesoreria_PowerQuery.xlsx
+++ b/libro/Tesoreria_PowerQuery.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6CBACED0-0569-4338-A185-05897EB42769}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81D883AA-4610-45B5-9C03-2D307664398F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-103" yWindow="-103" windowWidth="22149" windowHeight="13200" firstSheet="2" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-103" yWindow="-103" windowWidth="22149" windowHeight="13200" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Movimientos" sheetId="3" r:id="rId1"/>
@@ -25,7 +25,7 @@
   </definedNames>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="6" r:id="rId8"/>
+    <pivotCache cacheId="7" r:id="rId8"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -316,7 +316,7 @@
   </cellStyles>
   <dxfs count="8">
     <dxf>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+      <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
@@ -337,7 +337,7 @@
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
+      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
@@ -353,7 +353,7 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" refreshOnLoad="1" mc:Ignorable="xr" r:id="rId1" refreshedBy="Javier Angosto" refreshedDate="46324.46357777778" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="5" xr:uid="{450116B4-AE60-4FF3-861F-BEE85B5F3E92}">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="Javier Angosto" refreshedDate="46324.471488888892" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="5" xr:uid="{450116B4-AE60-4FF3-861F-BEE85B5F3E92}">
   <cacheSource type="worksheet">
     <worksheetSource name="PosiciónCaja"/>
   </cacheSource>
@@ -374,12 +374,12 @@
     </cacheField>
     <cacheField name="Saldo" numFmtId="0">
       <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" minValue="66250" maxValue="1256110.8500000001" count="6">
-        <n v="896580.65"/>
+        <n v="886580.65"/>
         <n v="1256110.8500000001"/>
         <n v="161665"/>
         <n v="469989.8"/>
         <n v="66250"/>
-        <n v="886580.65" u="1"/>
+        <n v="896580.65" u="1"/>
       </sharedItems>
     </cacheField>
     <cacheField name="Unidades_por_EUR" numFmtId="0">
@@ -404,7 +404,7 @@
     <x v="0"/>
     <x v="0"/>
     <n v="1"/>
-    <n v="896580.65"/>
+    <n v="886580.65"/>
   </r>
   <r>
     <x v="1"/>
@@ -438,7 +438,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{F4F508C4-12A7-45EC-A787-05AE7EE7717D}" name="TablaDinámica1" cacheId="6" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{F4F508C4-12A7-45EC-A787-05AE7EE7717D}" name="TablaDinámica1" cacheId="7" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="G3:H17" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="5">
     <pivotField axis="axisRow" showAll="0">
@@ -462,9 +462,9 @@
         <item x="4"/>
         <item x="2"/>
         <item x="3"/>
+        <item x="0"/>
+        <item x="1"/>
         <item m="1" x="5"/>
-        <item x="1"/>
-        <item x="0"/>
         <item t="default"/>
       </items>
     </pivotField>
@@ -484,7 +484,7 @@
       <x/>
     </i>
     <i r="2">
-      <x v="5"/>
+      <x v="3"/>
     </i>
     <i r="1">
       <x v="2"/>
@@ -612,10 +612,10 @@
     <sortCondition ref="A1:A26"/>
   </sortState>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{EE48C18E-21F0-4EF3-A363-563254CFDDD0}" uniqueName="1" name="Fecha" queryTableFieldId="1" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{EE48C18E-21F0-4EF3-A363-563254CFDDD0}" uniqueName="1" name="Fecha" queryTableFieldId="1" dataDxfId="7"/>
     <tableColumn id="2" xr3:uid="{859F7CBF-C07F-4FD6-8320-D85B973C7099}" uniqueName="2" name="Banco" queryTableFieldId="2"/>
     <tableColumn id="3" xr3:uid="{8809BD40-A305-4135-8DFF-15E539E76E47}" uniqueName="3" name="Cuenta" queryTableFieldId="3"/>
-    <tableColumn id="4" xr3:uid="{8FF8859E-42F1-4CC1-9CCA-486D1957BDCA}" uniqueName="4" name="Concepto" queryTableFieldId="4" dataDxfId="1"/>
+    <tableColumn id="4" xr3:uid="{8FF8859E-42F1-4CC1-9CCA-486D1957BDCA}" uniqueName="4" name="Concepto" queryTableFieldId="4" dataDxfId="6"/>
     <tableColumn id="5" xr3:uid="{C53DB4CA-7120-4B21-AD2C-B41CFD0D00BB}" uniqueName="5" name="Importe" queryTableFieldId="5"/>
     <tableColumn id="6" xr3:uid="{E921987E-58FF-42DB-A7DB-DE666F57D66F}" uniqueName="6" name="Divisa" queryTableFieldId="6"/>
   </tableColumns>
@@ -638,8 +638,8 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{C02CFB69-0B28-4221-95BB-8C8026A90067}" name="PosiciónCaja" displayName="PosiciónCaja" ref="A1:E7" tableType="queryTable" totalsRowCount="1">
   <autoFilter ref="A1:E6" xr:uid="{C02CFB69-0B28-4221-95BB-8C8026A90067}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{2CB0650B-143A-4854-A19B-29674EAE29E1}" uniqueName="1" name="Sociedad" totalsRowLabel="Total" queryTableFieldId="1" dataDxfId="7"/>
-    <tableColumn id="2" xr3:uid="{E1702D5A-7DE1-4365-AE26-A4BAED1EF381}" uniqueName="2" name="Divisa" queryTableFieldId="2" dataDxfId="6"/>
+    <tableColumn id="1" xr3:uid="{2CB0650B-143A-4854-A19B-29674EAE29E1}" uniqueName="1" name="Sociedad" totalsRowLabel="Total" queryTableFieldId="1" dataDxfId="5"/>
+    <tableColumn id="2" xr3:uid="{E1702D5A-7DE1-4365-AE26-A4BAED1EF381}" uniqueName="2" name="Divisa" queryTableFieldId="2" dataDxfId="4"/>
     <tableColumn id="3" xr3:uid="{2B950421-2F74-4BB5-9D5A-2916845DBCDE}" uniqueName="3" name="Saldo" queryTableFieldId="3"/>
     <tableColumn id="4" xr3:uid="{6577C2A1-C069-4A40-B786-87523BAEBE7C}" uniqueName="4" name="Unidades_por_EUR" queryTableFieldId="4"/>
     <tableColumn id="5" xr3:uid="{6BB5C8BB-9E4F-40B5-BF7E-AB7B30151A8E}" uniqueName="5" name="Saldo_EUR" totalsRowFunction="sum" queryTableFieldId="5"/>
@@ -652,10 +652,10 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{9737BECF-DD55-4155-9871-8B73DD3C64E8}" name="Saldos_Cuenta" displayName="Saldos_Cuenta" ref="A1:G6" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A1:G6" xr:uid="{9737BECF-DD55-4155-9871-8B73DD3C64E8}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{C1918784-1454-45F1-BA72-C16867338101}" uniqueName="1" name="Cuenta" queryTableFieldId="1" dataDxfId="5"/>
-    <tableColumn id="2" xr3:uid="{856BAEBC-6AF9-4768-B374-7ED36A26C084}" uniqueName="2" name="Banco" queryTableFieldId="2" dataDxfId="4"/>
-    <tableColumn id="3" xr3:uid="{F70630EC-488B-446C-A346-4FF18C436FA1}" uniqueName="3" name="Sociedad" queryTableFieldId="3" dataDxfId="3"/>
-    <tableColumn id="4" xr3:uid="{3BDF22D3-F4EA-4EFB-AA3E-88B0E7D59D77}" uniqueName="4" name="Divisa" queryTableFieldId="4" dataDxfId="2"/>
+    <tableColumn id="1" xr3:uid="{C1918784-1454-45F1-BA72-C16867338101}" uniqueName="1" name="Cuenta" queryTableFieldId="1" dataDxfId="3"/>
+    <tableColumn id="2" xr3:uid="{856BAEBC-6AF9-4768-B374-7ED36A26C084}" uniqueName="2" name="Banco" queryTableFieldId="2" dataDxfId="2"/>
+    <tableColumn id="3" xr3:uid="{F70630EC-488B-446C-A346-4FF18C436FA1}" uniqueName="3" name="Sociedad" queryTableFieldId="3" dataDxfId="1"/>
+    <tableColumn id="4" xr3:uid="{3BDF22D3-F4EA-4EFB-AA3E-88B0E7D59D77}" uniqueName="4" name="Divisa" queryTableFieldId="4" dataDxfId="0"/>
     <tableColumn id="5" xr3:uid="{2A680F31-08A6-49F6-BA0B-C280B6A2B848}" uniqueName="5" name="Saldo_inicial" queryTableFieldId="5"/>
     <tableColumn id="6" xr3:uid="{6B5C511C-8561-475D-BB39-B05D5026DA34}" uniqueName="6" name="Movimientos" queryTableFieldId="6"/>
     <tableColumn id="7" xr3:uid="{51DB7120-11B9-4E10-92C5-A2B13DCD1E46}" uniqueName="7" name="Saldo_Final" queryTableFieldId="7"/>
@@ -1684,7 +1684,7 @@
         <v>8</v>
       </c>
       <c r="H4" s="10">
-        <v>1045580.65</v>
+        <v>1035580.65</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.4">
@@ -1707,7 +1707,7 @@
         <v>9</v>
       </c>
       <c r="H5" s="10">
-        <v>896580.65</v>
+        <v>886580.65</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.4">
@@ -1727,10 +1727,10 @@
         <v>66250</v>
       </c>
       <c r="G6" s="9">
-        <v>896580.65</v>
+        <v>886580.65</v>
       </c>
       <c r="H6" s="10">
-        <v>896580.65</v>
+        <v>886580.65</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.4">
@@ -1825,7 +1825,7 @@
         <v>52</v>
       </c>
       <c r="H17" s="10">
-        <v>2827719.16</v>
+        <v>2817719.16</v>
       </c>
     </row>
   </sheetData>

</xml_diff>